<commit_message>
Working on BXCC stuff
</commit_message>
<xml_diff>
--- a/data/HeatLossFlows.xlsx
+++ b/data/HeatLossFlows.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/MaterialExergyPaper2025/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C13A21F-7860-5149-9A91-E9BADD1325E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC4CFF9-490D-6245-8BAC-4254A7EA2F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23060" yWindow="4340" windowWidth="28040" windowHeight="17440" xr2:uid="{742590E8-047E-1447-91ED-17B8D0993C1D}"/>
+    <workbookView xWindow="19180" yWindow="3060" windowWidth="28040" windowHeight="17440" xr2:uid="{742590E8-047E-1447-91ED-17B8D0993C1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,51 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Matt</author>
+  </authors>
+  <commentList>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{E36F0B66-EA10-EC4E-8916-486EEA2766FB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Matt:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Temperatures below the line are all from the BXCC Q loss tab in the Paper Examples.xlsx file.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
   <si>
     <t>Industry</t>
   </si>
@@ -149,9 +192,6 @@
     <t>COG treatment</t>
   </si>
   <si>
-    <t>HTH.2373.K</t>
-  </si>
-  <si>
     <t>HeatLossFlow</t>
   </si>
   <si>
@@ -164,9 +204,6 @@
     <t>https://pelletindia.com/blog/2024/09/11/charcoal-carbonization-and-torrefaction-of-biomass-materials-relate-to-their-processing-temperatures-chemical-properties-and-end-uses/</t>
   </si>
   <si>
-    <t>https://ifrf.net/research/handbook/what-are-the-combustion-and-flue-gas-properties-of-coke-oven-gas/#:~:text=The%20high%20hydrogen%20concentration%20in,gas%20flame%20at%20stoichiometric%20conditions.</t>
-  </si>
-  <si>
     <t>https://www.economics.utoronto.ca/munro5/BlastFurnaceHydraulic.pdf</t>
   </si>
   <si>
@@ -200,9 +237,6 @@
     <t>Assumed exhaust temperature</t>
   </si>
   <si>
-    <t>HTH.1173.K</t>
-  </si>
-  <si>
     <t>**** Need to decide a temperature</t>
   </si>
   <si>
@@ -210,13 +244,31 @@
   </si>
   <si>
     <t>TemperatureK</t>
+  </si>
+  <si>
+    <t>HTH.1175.C</t>
+  </si>
+  <si>
+    <t>HTH.900.C</t>
+  </si>
+  <si>
+    <t>HTH.1300.C</t>
+  </si>
+  <si>
+    <t>HTH.2100.C</t>
+  </si>
+  <si>
+    <t>LTH.65.C</t>
+  </si>
+  <si>
+    <t>LTH.50.C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -231,6 +283,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -611,7 +676,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA1AC2A6-D39E-A444-B5A1-5D796C28F5AC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA1AC2A6-D39E-A444-B5A1-5D796C28F5AC}">
   <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -625,16 +690,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -652,7 +717,7 @@
         <v>0.73937937062937065</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -660,7 +725,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <f>600+273.15</f>
@@ -671,7 +736,7 @@
         <v>0.65853518868464755</v>
       </c>
       <c r="E3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -679,7 +744,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4">
         <f>500+273.15</f>
@@ -690,7 +755,7 @@
         <v>0.61436978594063252</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -698,7 +763,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5">
         <f>2500+273.15</f>
@@ -709,7 +774,7 @@
         <v>0.8924868831473235</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -727,7 +792,7 @@
         <v>0.81045772409408778</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -735,7 +800,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C7">
         <f>25+273.15</f>
@@ -746,7 +811,7 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -754,7 +819,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C8">
         <f>(1200-32)*5/9 + 273.15</f>
@@ -765,7 +830,7 @@
         <v>0.67664053697421778</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -773,7 +838,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <f>200+273.15</f>
@@ -784,7 +849,7 @@
         <v>0.36986156609954557</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -792,7 +857,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C10">
         <f t="shared" ref="C10:C20" si="1">25+273.15</f>
@@ -808,7 +873,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C11">
         <f t="shared" si="1"/>
@@ -824,7 +889,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C12">
         <f t="shared" si="1"/>
@@ -840,7 +905,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C13">
         <f t="shared" si="1"/>
@@ -856,7 +921,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C14">
         <f t="shared" si="1"/>
@@ -872,7 +937,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C15">
         <f t="shared" si="1"/>
@@ -888,7 +953,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16">
         <f>2500+273.15</f>
@@ -899,7 +964,7 @@
         <v>0.8924868831473235</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -907,7 +972,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17">
         <f t="shared" si="1"/>
@@ -923,7 +988,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C18">
         <f>2500+273.15</f>
@@ -934,7 +999,7 @@
         <v>0.8924868831473235</v>
       </c>
       <c r="E18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -942,7 +1007,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C19">
         <f>2500+273.15</f>
@@ -953,7 +1018,7 @@
         <v>0.8924868831473235</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -961,7 +1026,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C20">
         <f t="shared" si="1"/>
@@ -977,18 +1042,14 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="C21">
-        <f t="shared" ref="C21:C29" si="2">2500+273.15</f>
-        <v>2773.15</v>
+        <v>338.15</v>
       </c>
       <c r="D21">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E21" t="s">
-        <v>49</v>
+        <v>0.11829069939376013</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -996,18 +1057,14 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C22">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>323.14999999999998</v>
       </c>
       <c r="D22">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E22" t="s">
-        <v>49</v>
+        <v>7.7363453504564417E-2</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1015,18 +1072,14 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C23">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>323.14999999999998</v>
       </c>
       <c r="D23">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E23" t="s">
-        <v>49</v>
+        <v>7.7363453504564417E-2</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1034,18 +1087,14 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C24">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D24">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E24" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1053,18 +1102,14 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C25">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D25">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E25" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1072,18 +1117,14 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C26">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D26">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E26" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1091,18 +1132,14 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C27">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>1448.15</v>
       </c>
       <c r="D27">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E27" t="s">
-        <v>49</v>
+        <v>0.79411663156440981</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1110,18 +1147,14 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C28">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D28">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E28" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1129,18 +1162,14 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C29">
-        <f t="shared" si="2"/>
-        <v>2773.15</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D29">
         <f t="shared" si="0"/>
-        <v>0.8924868831473235</v>
-      </c>
-      <c r="E29" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1148,14 +1177,14 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C30">
-        <v>1173</v>
+        <v>1173.1500000000001</v>
       </c>
       <c r="D30">
         <f t="shared" si="0"/>
-        <v>0.74582267689684567</v>
+        <v>0.74585517623492303</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1163,62 +1192,55 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C31">
-        <v>1573</v>
+        <v>1573.15</v>
       </c>
       <c r="D31">
         <f t="shared" si="0"/>
-        <v>0.81045772409408778</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>44</v>
-      </c>
+        <v>0.81047579696786709</v>
+      </c>
+      <c r="E31" s="3"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C32">
-        <f t="shared" ref="C32:C34" si="3">25+273.15</f>
-        <v>298.14999999999998</v>
+        <v>2373.15</v>
       </c>
       <c r="D32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.87436529507195082</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C33">
-        <v>2373</v>
+        <v>298.14999999999998</v>
       </c>
       <c r="D33">
         <f t="shared" si="0"/>
-        <v>0.87435735356089339</v>
-      </c>
-      <c r="E33" t="s">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C34">
-        <f t="shared" si="3"/>
         <v>298.14999999999998</v>
       </c>
       <c r="D34">
@@ -1241,16 +1263,16 @@
         <v>0.73937937062937065</v>
       </c>
       <c r="E35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E6" r:id="rId1" xr:uid="{C8BF8FD3-09EB-A24C-96AE-02A6FAC1C1FB}"/>
-    <hyperlink ref="E31" r:id="rId2" xr:uid="{235A2FDB-7FDE-2447-A2D4-4CD848ECE1AB}"/>
-    <hyperlink ref="E8" r:id="rId3" xr:uid="{2018C0C2-0D95-AA4A-81A8-86F9B4FF2499}"/>
+    <hyperlink ref="E8" r:id="rId2" xr:uid="{2018C0C2-0D95-AA4A-81A8-86F9B4FF2499}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>